<commit_message>
Updating the model for Rosiori
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Consumption_Forecast.xlsx
+++ b/data_fetching/Entsoe/Consumption_Forecast.xlsx
@@ -394,770 +394,770 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="B2">
-        <v>4820</v>
+        <v>4720</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46299.01041666666</v>
+        <v>46300.01041666666</v>
       </c>
       <c r="B3">
-        <v>4770</v>
+        <v>4680</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46299.02083333334</v>
+        <v>46300.02083333334</v>
       </c>
       <c r="B4">
-        <v>4720</v>
+        <v>4650</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46299.03125</v>
+        <v>46300.03125</v>
       </c>
       <c r="B5">
-        <v>4690</v>
+        <v>4630</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46299.04166666666</v>
+        <v>46300.04166666666</v>
       </c>
       <c r="B6">
-        <v>4640</v>
+        <v>4610</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46299.05208333334</v>
+        <v>46300.05208333334</v>
       </c>
       <c r="B7">
-        <v>4610</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46299.0625</v>
+        <v>46300.0625</v>
       </c>
       <c r="B8">
-        <v>4590</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46299.07291666666</v>
+        <v>46300.07291666666</v>
       </c>
       <c r="B9">
-        <v>4560</v>
+        <v>4610</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46299.08333333334</v>
+        <v>46300.08333333334</v>
       </c>
       <c r="B10">
-        <v>4540</v>
+        <v>4630</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46299.09375</v>
+        <v>46300.09375</v>
       </c>
       <c r="B11">
-        <v>4530</v>
+        <v>4650</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46299.10416666666</v>
+        <v>46300.10416666666</v>
       </c>
       <c r="B12">
-        <v>4530</v>
+        <v>4690</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46299.11458333334</v>
+        <v>46300.11458333334</v>
       </c>
       <c r="B13">
-        <v>4520</v>
+        <v>4720</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46299.125</v>
+        <v>46300.125</v>
       </c>
       <c r="B14">
-        <v>4500</v>
+        <v>4750</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46299.13541666666</v>
+        <v>46300.13541666666</v>
       </c>
       <c r="B15">
-        <v>4490</v>
+        <v>4790</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46299.14583333334</v>
+        <v>46300.14583333334</v>
       </c>
       <c r="B16">
-        <v>4500</v>
+        <v>4830</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46299.15625</v>
+        <v>46300.15625</v>
       </c>
       <c r="B17">
-        <v>4510</v>
+        <v>4890</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46299.16666666666</v>
+        <v>46300.16666666666</v>
       </c>
       <c r="B18">
-        <v>4550</v>
+        <v>4950</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46299.17708333334</v>
+        <v>46300.17708333334</v>
       </c>
       <c r="B19">
-        <v>4570</v>
+        <v>5040</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46299.1875</v>
+        <v>46300.1875</v>
       </c>
       <c r="B20">
-        <v>4590</v>
+        <v>5140</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46299.19791666666</v>
+        <v>46300.19791666666</v>
       </c>
       <c r="B21">
-        <v>4610</v>
+        <v>5270</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46299.20833333334</v>
+        <v>46300.20833333334</v>
       </c>
       <c r="B22">
-        <v>4650</v>
+        <v>5420</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46299.21875</v>
+        <v>46300.21875</v>
       </c>
       <c r="B23">
-        <v>4670</v>
+        <v>5580</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46299.22916666666</v>
+        <v>46300.22916666666</v>
       </c>
       <c r="B24">
-        <v>4690</v>
+        <v>5750</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46299.23958333334</v>
+        <v>46300.23958333334</v>
       </c>
       <c r="B25">
-        <v>4710</v>
+        <v>5910</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46299.25</v>
+        <v>46300.25</v>
       </c>
       <c r="B26">
-        <v>4740</v>
+        <v>6050</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46299.26041666666</v>
+        <v>46300.26041666666</v>
       </c>
       <c r="B27">
-        <v>4760</v>
+        <v>6180</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46299.27083333334</v>
+        <v>46300.27083333334</v>
       </c>
       <c r="B28">
-        <v>4760</v>
+        <v>6270</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46299.28125</v>
+        <v>46300.28125</v>
       </c>
       <c r="B29">
-        <v>4740</v>
+        <v>6300</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46299.29166666666</v>
+        <v>46300.29166666666</v>
       </c>
       <c r="B30">
-        <v>4720</v>
+        <v>6290</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46299.30208333334</v>
+        <v>46300.30208333334</v>
       </c>
       <c r="B31">
-        <v>4690</v>
+        <v>6270</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46299.3125</v>
+        <v>46300.3125</v>
       </c>
       <c r="B32">
-        <v>4640</v>
+        <v>6210</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46299.32291666666</v>
+        <v>46300.32291666666</v>
       </c>
       <c r="B33">
-        <v>4550</v>
+        <v>6090</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46299.33333333334</v>
+        <v>46300.33333333334</v>
       </c>
       <c r="B34">
-        <v>4370</v>
+        <v>5940</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46299.34375</v>
+        <v>46300.34375</v>
       </c>
       <c r="B35">
-        <v>4210</v>
+        <v>5770</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46299.35416666666</v>
+        <v>46300.35416666666</v>
       </c>
       <c r="B36">
-        <v>4060</v>
+        <v>5580</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46299.36458333334</v>
+        <v>46300.36458333334</v>
       </c>
       <c r="B37">
-        <v>3920</v>
+        <v>5380</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46299.375</v>
+        <v>46300.375</v>
       </c>
       <c r="B38">
-        <v>3790</v>
+        <v>5190</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46299.38541666666</v>
+        <v>46300.38541666666</v>
       </c>
       <c r="B39">
-        <v>3660</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46299.39583333334</v>
+        <v>46300.39583333334</v>
       </c>
       <c r="B40">
-        <v>3500</v>
+        <v>4820</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46299.40625</v>
+        <v>46300.40625</v>
       </c>
       <c r="B41">
-        <v>3370</v>
+        <v>4670</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46299.41666666666</v>
+        <v>46300.41666666666</v>
       </c>
       <c r="B42">
-        <v>3220</v>
+        <v>4530</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46299.42708333334</v>
+        <v>46300.42708333334</v>
       </c>
       <c r="B43">
-        <v>3110</v>
+        <v>4420</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46299.4375</v>
+        <v>46300.4375</v>
       </c>
       <c r="B44">
-        <v>3050</v>
+        <v>4330</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46299.44791666666</v>
+        <v>46300.44791666666</v>
       </c>
       <c r="B45">
-        <v>3020</v>
+        <v>4260</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46299.45833333334</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="B46">
-        <v>3000</v>
+        <v>4220</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46299.46875</v>
+        <v>46300.46875</v>
       </c>
       <c r="B47">
-        <v>2990</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46299.47916666666</v>
+        <v>46300.47916666666</v>
       </c>
       <c r="B48">
-        <v>2990</v>
+        <v>4190</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46299.48958333334</v>
+        <v>46300.48958333334</v>
       </c>
       <c r="B49">
-        <v>3020</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46299.5</v>
+        <v>46300.5</v>
       </c>
       <c r="B50">
-        <v>3050</v>
+        <v>4220</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46299.51041666666</v>
+        <v>46300.51041666666</v>
       </c>
       <c r="B51">
-        <v>3080</v>
+        <v>4240</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46299.52083333334</v>
+        <v>46300.52083333334</v>
       </c>
       <c r="B52">
-        <v>3110</v>
+        <v>4260</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46299.53125</v>
+        <v>46300.53125</v>
       </c>
       <c r="B53">
-        <v>3160</v>
+        <v>4290</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46299.54166666666</v>
+        <v>46300.54166666666</v>
       </c>
       <c r="B54">
-        <v>3210</v>
+        <v>4320</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46299.55208333334</v>
+        <v>46300.55208333334</v>
       </c>
       <c r="B55">
-        <v>3270</v>
+        <v>4360</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46299.5625</v>
+        <v>46300.5625</v>
       </c>
       <c r="B56">
-        <v>3330</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46299.57291666666</v>
+        <v>46300.57291666666</v>
       </c>
       <c r="B57">
-        <v>3390</v>
+        <v>4460</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46299.58333333334</v>
+        <v>46300.58333333334</v>
       </c>
       <c r="B58">
-        <v>3450</v>
+        <v>4520</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46299.59375</v>
+        <v>46300.59375</v>
       </c>
       <c r="B59">
-        <v>3510</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46299.60416666666</v>
+        <v>46300.60416666666</v>
       </c>
       <c r="B60">
-        <v>3580</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46299.61458333334</v>
+        <v>46300.61458333334</v>
       </c>
       <c r="B61">
-        <v>3660</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46299.625</v>
+        <v>46300.625</v>
       </c>
       <c r="B62">
-        <v>3750</v>
+        <v>4920</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46299.63541666666</v>
+        <v>46300.63541666666</v>
       </c>
       <c r="B63">
-        <v>3870</v>
+        <v>5050</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46299.64583333334</v>
+        <v>46300.64583333334</v>
       </c>
       <c r="B64">
-        <v>4010</v>
+        <v>5180</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46299.65625</v>
+        <v>46300.65625</v>
       </c>
       <c r="B65">
-        <v>4170</v>
+        <v>5330</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46299.66666666666</v>
+        <v>46300.66666666666</v>
       </c>
       <c r="B66">
-        <v>4380</v>
+        <v>5470</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46299.67708333334</v>
+        <v>46300.67708333334</v>
       </c>
       <c r="B67">
-        <v>4560</v>
+        <v>5630</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46299.6875</v>
+        <v>46300.6875</v>
       </c>
       <c r="B68">
-        <v>4740</v>
+        <v>5780</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46299.69791666666</v>
+        <v>46300.69791666666</v>
       </c>
       <c r="B69">
-        <v>4920</v>
+        <v>5940</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46299.70833333334</v>
+        <v>46300.70833333334</v>
       </c>
       <c r="B70">
-        <v>5090</v>
+        <v>6090</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46299.71875</v>
+        <v>46300.71875</v>
       </c>
       <c r="B71">
-        <v>5230</v>
+        <v>6230</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46299.72916666666</v>
+        <v>46300.72916666666</v>
       </c>
       <c r="B72">
-        <v>5370</v>
+        <v>6360</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46299.73958333334</v>
+        <v>46300.73958333334</v>
       </c>
       <c r="B73">
-        <v>5510</v>
+        <v>6480</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46299.75</v>
+        <v>46300.75</v>
       </c>
       <c r="B74">
-        <v>5670</v>
+        <v>6590</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46299.76041666666</v>
+        <v>46300.76041666666</v>
       </c>
       <c r="B75">
-        <v>5810</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46299.77083333334</v>
+        <v>46300.77083333334</v>
       </c>
       <c r="B76">
-        <v>5920</v>
+        <v>6810</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46299.78125</v>
+        <v>46300.78125</v>
       </c>
       <c r="B77">
-        <v>6000</v>
+        <v>6910</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46299.79166666666</v>
+        <v>46300.79166666666</v>
       </c>
       <c r="B78">
-        <v>6050</v>
+        <v>7010</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46299.80208333334</v>
+        <v>46300.80208333334</v>
       </c>
       <c r="B79">
-        <v>6070</v>
+        <v>7050</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46299.8125</v>
+        <v>46300.8125</v>
       </c>
       <c r="B80">
-        <v>6060</v>
+        <v>7030</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46299.82291666666</v>
+        <v>46300.82291666666</v>
       </c>
       <c r="B81">
-        <v>6020</v>
+        <v>6940</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46299.83333333334</v>
+        <v>46300.83333333334</v>
       </c>
       <c r="B82">
-        <v>5900</v>
+        <v>6720</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46299.84375</v>
+        <v>46300.84375</v>
       </c>
       <c r="B83">
-        <v>5750</v>
+        <v>6480</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46299.85416666666</v>
+        <v>46300.85416666666</v>
       </c>
       <c r="B84">
-        <v>5620</v>
+        <v>6360</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46299.86458333334</v>
+        <v>46300.86458333334</v>
       </c>
       <c r="B85">
-        <v>5530</v>
+        <v>6310</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46299.875</v>
+        <v>46300.875</v>
       </c>
       <c r="B86">
-        <v>5420</v>
+        <v>6220</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46299.88541666666</v>
+        <v>46300.88541666666</v>
       </c>
       <c r="B87">
-        <v>5340</v>
+        <v>6100</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46299.89583333334</v>
+        <v>46300.89583333334</v>
       </c>
       <c r="B88">
-        <v>5260</v>
+        <v>5880</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46299.90625</v>
+        <v>46300.90625</v>
       </c>
       <c r="B89">
-        <v>5180</v>
+        <v>5800</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46299.91666666666</v>
+        <v>46300.91666666666</v>
       </c>
       <c r="B90">
-        <v>5090</v>
+        <v>5750</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46299.92708333334</v>
+        <v>46300.92708333334</v>
       </c>
       <c r="B91">
-        <v>5010</v>
+        <v>5670</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46299.9375</v>
+        <v>46300.9375</v>
       </c>
       <c r="B92">
-        <v>4960</v>
+        <v>5620</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46299.94791666666</v>
+        <v>46300.94791666666</v>
       </c>
       <c r="B93">
-        <v>4940</v>
+        <v>5530</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46299.95833333334</v>
+        <v>46300.95833333334</v>
       </c>
       <c r="B94">
-        <v>4920</v>
+        <v>5530</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46299.96875</v>
+        <v>46300.96875</v>
       </c>
       <c r="B95">
-        <v>4900</v>
+        <v>5530</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46299.97916666666</v>
+        <v>46300.97916666666</v>
       </c>
       <c r="B96">
-        <v>4840</v>
+        <v>5530</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46299.98958333334</v>
+        <v>46300.98958333334</v>
       </c>
       <c r="B97">
-        <v>4770</v>
+        <v>5530</v>
       </c>
     </row>
   </sheetData>

</xml_diff>